<commit_message>
Add Piyush Shukla, Dr. Eka Devidze, and Assoc. Prof. Dr. Muliati Hj. Sedek to AIFORGE 2026 keynote speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,13 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="55.83203125" customWidth="1"/>
-    <col min="5" max="5" width="85.83203125" customWidth="1"/>
+    <col min="4" max="4" width="65.83203125" customWidth="1"/>
+    <col min="5" max="5" width="95.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
@@ -583,18 +583,41 @@
         <v>Add Parikshit Sahagal to AIFORGE 2026</v>
       </c>
       <c r="E8" t="str">
-        <v>Added Parikshit Sahagal (Technical Project Manager, CoStar Group Inc, USA) as Keynote Speaker with official portrait.</v>
+        <v>Added Parikshit Sahagal (Technical Project Manager, CoStar Group Inc, USA) as Keynote Speaker with official portrait, positioned between Dr. Peter Kamau and Jaco Visagie.</v>
       </c>
       <c r="F8" t="str">
         <v>Completed</v>
       </c>
       <c r="G8" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Keynote Speakers</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Add Piyush Shukla, Dr. Eka Devidze &amp; Assoc. Prof. Dr. Muliati Hj. Sedek to AIFORGE 2026</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Added Piyush Shukla (Technology &amp; Engineering Leader, USA), Dr. Eka Devidze (Affiliated Professor, The University of Georgia, Georgia), and Assoc. Prof. Dr. Muliati Hj. Sedek (Deputy Director CAES, UTeM Malaysia) to AIFORGE 2026 with official portraits.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G9" t="str">
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sandeep Kumar Khandelwal and Prof. Rehab Hegazy to AIFORGE 2026 invited speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -615,9 +615,55 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Invited Speakers</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Add Assoc. Prof. Ts. Dr. Noor Suhana Binti Sulaiman to AIFORGE 2026</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Added Assoc. Prof. Ts. Dr. Noor Suhana Binti Sulaiman (Dean, Research &amp; Postgraduate Management, University College TATI, Malaysia) as Invited Speaker.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G10" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Invited Speakers</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Add Sandeep Kumar Khandelwal &amp; Prof. Rehab Hegazy, PhD to AIFORGE 2026</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Added Sandeep Kumar Khandelwal (AI, DevOps &amp; Cloud Computing Expert, USA) and Prof. Rehab Hegazy, PhD (Professor of Pharmacology &amp; Secretary-General, NRC Egypt) as Invited Speakers.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G11" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Prof. Intakhab Alam Khan and Osman ARAYICI to AIFORGE 2026 invited speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -661,9 +661,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Invited Speakers</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Add Prof. Intakhab Alam Khan &amp; Osman ARAYICI to AIFORGE 2026</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Added Prof. Intakhab Alam Khan (King Abdulaziz University, Saudi Arabia &amp; Samarkand State University) and Osman ARAYICI (Mimar Sinan Fine Arts University / Modoko Academy, Turkey) as Invited Speakers.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G12" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Swarnabindu Roy, Payal R., and Dr. Carolina Barandiaran to AIFORGE 2026 keynote speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -684,9 +684,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Keynote Speakers</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Add Swarnabindu Roy, Payal R. &amp; Dr. Carolina Barandiaran to AIFORGE 2026</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Added Swarnabindu Roy (Data Engineering &amp; Program Management, USA), Payal R. (Senior Data Engineer, ETL Pipelines, USA), and Dr. Carolina Barandiaran (Academic Leader &amp; Researcher, Argentina) as Keynote Speakers.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G13" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move Marghescu Cristina-Florentina, Nadine Zeinoun, Dr. Mbombi Khizamane, and Dr. Tintin Flores to Advisory Board Members and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -707,9 +707,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Advisory Board</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Move 4 Speakers to Advisory Board Members in AIFORGE 2026</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Moved Marghescu Cristina-Florentina, Nadine Zeinoun, Dr. Mbombi Khizamane, and Dr. Tintin Flores from Speakers section to Advisory Board Members section with Advisory Board Member title.</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G14" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Swarnabindu Roy photo and remove Iterative International Publishers (IIP) from AIFORGE 2026
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -730,9 +730,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Publications / Keynote</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Update Swarnabindu Roy Photo &amp; Remove IIP from Publications</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Updated Swarnabindu Roy's portrait photo to executive boardroom portrait and removed Iterative International Publishers (IIP) from AIFORGE 2026 Publications section.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G15" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Nino Devidze and Lali Mikeladze to AIFORGE 2026 distinguished speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -753,9 +753,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Distinguished Speakers</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Add Nino Devidze &amp; Lali Mikeladze to AIFORGE 2026</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Added Nino Devidze (Tourism Educator &amp; Program Manager, The University of Georgia) and Lali Mikeladze (Head of the BA Program in Tourism, Caucasus International University, Georgia) as Distinguished Speakers with official portraits.</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G16" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Create 3-part Instagram post flyers for AIFORGE 2026 speakers and update Daily Work Records
</commit_message>
<xml_diff>
--- a/Daily Work Records.xlsx
+++ b/Daily Work Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -776,9 +776,32 @@
         <v>main (Kddee/conference-hubbb)</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Social Media / Flyers</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Create 3-Part Instagram Post Carousel Flyers for AIFORGE 2026 Speakers</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Designed and developed a 3-part Instagram post flyer set (1080x1350 px, 4:5 vertical portrait) featuring all 22 conference speakers divided across 3 flyers (excluding Prof. Dr. Alexander Bull), with conference branding, titles, designations, ISBN, date, QR code, and 1-click high-resolution PNG export.</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="G17" t="str">
+        <v>main (Kddee/conference-hubbb)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>